<commit_message>
Updated spreadsheet and script to reflect new payment amounts that will start in November 2026
</commit_message>
<xml_diff>
--- a/Student_Loan_Payoff_Dashboard.xlsx
+++ b/Student_Loan_Payoff_Dashboard.xlsx
@@ -604,11 +604,11 @@
         </c:ser>
         <c:gapWidth val="150"/>
         <c:overlap val="0"/>
-        <c:axId val="2276864"/>
-        <c:axId val="79511964"/>
+        <c:axId val="81174393"/>
+        <c:axId val="3034470"/>
       </c:barChart>
       <c:catAx>
-        <c:axId val="2276864"/>
+        <c:axId val="81174393"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -674,7 +674,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="79511964"/>
+        <c:crossAx val="3034470"/>
         <c:crosses val="autoZero"/>
         <c:auto val="1"/>
         <c:lblAlgn val="ctr"/>
@@ -682,7 +682,7 @@
         <c:noMultiLvlLbl val="0"/>
       </c:catAx>
       <c:valAx>
-        <c:axId val="79511964"/>
+        <c:axId val="3034470"/>
         <c:scaling>
           <c:orientation val="minMax"/>
         </c:scaling>
@@ -758,7 +758,7 @@
             </a:pPr>
           </a:p>
         </c:txPr>
-        <c:crossAx val="2276864"/>
+        <c:crossAx val="81174393"/>
         <c:crosses val="autoZero"/>
         <c:crossBetween val="between"/>
       </c:valAx>

</xml_diff>